<commit_message>
Cadastro: regime de 78 clientes que estavam em branco
Simples (6) e MEI (8) pela opção cadastral na Receita (BrasilAPI,
consulta pública por CNPJ); Física (64) por serem CPF. Ficam em branco
só os que a Receita não define: 391 (excluída do Simples em 2024,
ativa), 426 e 480 (baixadas) e a linha de modelo 1.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/necessario para o claude/dados agentes/cadastro_empresas_unificado.xlsx
+++ b/necessario para o claude/dados agentes/cadastro_empresas_unificado.xlsx
@@ -571,6 +571,11 @@
           <t>03838458153</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -596,6 +601,11 @@
           <t>03838413128</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -696,6 +706,11 @@
           <t>03899406620</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1126,6 +1141,11 @@
           <t>03838453284</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1356,6 +1376,11 @@
           <t>03891341653</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1581,6 +1606,11 @@
           <t>3838452074</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1936,6 +1966,11 @@
           <t>03838321385</t>
         </is>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1961,6 +1996,11 @@
           <t>03838451510</t>
         </is>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -2191,6 +2231,11 @@
           <t>001648660.00-80</t>
         </is>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -2216,6 +2261,11 @@
           <t>03838451593</t>
         </is>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -2791,6 +2841,11 @@
           <t>03899499121</t>
         </is>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2956,6 +3011,11 @@
           <t>03838451859</t>
         </is>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -3021,6 +3081,11 @@
           <t>0032125710013</t>
         </is>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -3216,6 +3281,11 @@
           <t>003331622.00-89</t>
         </is>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -3246,6 +3316,11 @@
           <t>003337496.00-14</t>
         </is>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -3276,6 +3351,11 @@
           <t>003184443.00-73</t>
         </is>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -3306,6 +3386,11 @@
           <t>003279501.00-89</t>
         </is>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -3336,6 +3421,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -3366,6 +3456,11 @@
           <t>0030641430086</t>
         </is>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -3396,6 +3491,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -3426,6 +3526,11 @@
           <t>003183541.00-90</t>
         </is>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -3491,6 +3596,11 @@
           <t>003129382.00-59</t>
         </is>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -3521,6 +3631,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -3551,6 +3666,11 @@
           <t>003184458.00-59</t>
         </is>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -3581,6 +3701,11 @@
           <t>002811481.00-92</t>
         </is>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3611,6 +3736,11 @@
           <t>002278271.00-01</t>
         </is>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3641,6 +3771,11 @@
           <t>002291479.00-23</t>
         </is>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3671,6 +3806,11 @@
           <t>002493376.00-63</t>
         </is>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3701,6 +3841,11 @@
           <t>002465651.00-68</t>
         </is>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3731,6 +3876,11 @@
           <t>002208142.00-82</t>
         </is>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3761,6 +3911,11 @@
           <t>001721656.00-60</t>
         </is>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -3791,6 +3946,11 @@
           <t>003059849.00-78</t>
         </is>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -3821,6 +3981,11 @@
           <t>002087422.00-09</t>
         </is>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -3851,6 +4016,11 @@
           <t>03838451071</t>
         </is>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -3951,6 +4121,11 @@
           <t>002594616.00-36</t>
         </is>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -4016,6 +4191,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -4111,6 +4291,11 @@
           <t>0033857380071</t>
         </is>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -4141,6 +4326,11 @@
           <t>0033857530065</t>
         </is>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -4196,6 +4386,11 @@
           <t>03898360725</t>
         </is>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -4436,6 +4631,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -4566,6 +4766,11 @@
           <t>0035695690048</t>
         </is>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -4626,6 +4831,11 @@
           <t>0035942240051</t>
         </is>
       </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -4651,6 +4861,11 @@
           <t>0036353530030</t>
         </is>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -4676,6 +4891,11 @@
           <t>03891537487</t>
         </is>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -4701,6 +4921,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -4726,6 +4951,11 @@
           <t>03899727332</t>
         </is>
       </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -4821,6 +5051,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -4851,6 +5086,11 @@
           <t>0036793410059</t>
         </is>
       </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -4881,6 +5121,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -4911,6 +5156,11 @@
           <t>002261694.00-27</t>
         </is>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -4941,6 +5191,11 @@
           <t>3891517154</t>
         </is>
       </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -5036,6 +5291,11 @@
           <t>003716396.00-42</t>
         </is>
       </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -5236,6 +5496,11 @@
           <t>0037397770088</t>
         </is>
       </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -5261,6 +5526,11 @@
           <t>003756880.00-83</t>
         </is>
       </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -5291,6 +5561,11 @@
           <t>003758306.00-28</t>
         </is>
       </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -5316,6 +5591,11 @@
           <t>003763327.00-12</t>
         </is>
       </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -5341,6 +5621,11 @@
           <t>003758810.00-36</t>
         </is>
       </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -5366,6 +5651,11 @@
           <t>ISENTO</t>
         </is>
       </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -5396,6 +5686,11 @@
           <t>03891427184</t>
         </is>
       </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -5426,6 +5721,11 @@
           <t>03892429028</t>
         </is>
       </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -5811,6 +6111,11 @@
           <t>16981238998</t>
         </is>
       </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -5841,6 +6146,11 @@
           <t>003891547.00-95</t>
         </is>
       </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -6021,6 +6331,11 @@
           <t>3888522571</t>
         </is>
       </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>MEI</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -6191,6 +6506,11 @@
           <t>0039603140007</t>
         </is>
       </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -6221,6 +6541,11 @@
           <t>0039914900011</t>
         </is>
       </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -6251,6 +6576,11 @@
           <t>0039599540069</t>
         </is>
       </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -6316,6 +6646,11 @@
           <t>003160715.00-69</t>
         </is>
       </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -7116,6 +7451,11 @@
           <t>02195075500</t>
         </is>
       </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="n">
@@ -7176,6 +7516,11 @@
           <t>03899740018</t>
         </is>
       </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="n">
@@ -7276,6 +7621,11 @@
           <t>004105944.00-91</t>
         </is>
       </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="n">
@@ -9176,6 +9526,11 @@
           <t>3898613335</t>
         </is>
       </c>
+      <c r="G272" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" t="n">
@@ -9676,6 +10031,11 @@
           <t>03185343468</t>
         </is>
       </c>
+      <c r="G287" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
     </row>
     <row r="288">
       <c r="A288" t="n">
@@ -9876,6 +10236,11 @@
           <t>38998334460</t>
         </is>
       </c>
+      <c r="G293" t="inlineStr">
+        <is>
+          <t>Física</t>
+        </is>
+      </c>
     </row>
     <row r="294">
       <c r="A294" t="n">
@@ -10491,6 +10856,11 @@
           <t>3892571903</t>
         </is>
       </c>
+      <c r="G311" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" t="n">
@@ -10521,6 +10891,11 @@
           <t>3891802575</t>
         </is>
       </c>
+      <c r="G312" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" t="n">
@@ -10551,6 +10926,11 @@
           <t>(38)9881088</t>
         </is>
       </c>
+      <c r="G313" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" t="n">
@@ -10581,6 +10961,11 @@
           <t>3892168998</t>
         </is>
       </c>
+      <c r="G314" t="inlineStr">
+        <is>
+          <t>Simples</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" t="n">
@@ -10609,6 +10994,11 @@
       <c r="F315" t="inlineStr">
         <is>
           <t>3838458153</t>
+        </is>
+      </c>
+      <c r="G315" t="inlineStr">
+        <is>
+          <t>Física</t>
         </is>
       </c>
     </row>

</xml_diff>